<commit_message>
Corrected after further review of PR notes.
</commit_message>
<xml_diff>
--- a/Method Lists/Modus2 Soil Code Supersession.xlsx
+++ b/Method Lists/Modus2 Soil Code Supersession.xlsx
@@ -8,19 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aggateway-my.sharepoint.com/personal/ben_craker_aggateway_org/Documents/Working Groups/Agrisemantics Committee/Modus Source of Truth/Claude's Folder/Modus/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_B830711B1369A26F60327C7441B1DE79D657DCFF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_B830711B1369A26F60327C7441B1DE79D657DCFF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F580601E-FAFB-451A-89F2-83910ED6C26C}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$B$1032</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2064" uniqueCount="1756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2050" uniqueCount="1749">
   <si>
     <t>Modus Code (V1 &amp; V2)</t>
   </si>
@@ -3380,27 +3396,6 @@
   </si>
   <si>
     <t>L_MODV2_SOIL_TKN_007</t>
-  </si>
-  <si>
-    <t>L_MODV2_SOIL_TKN_008</t>
-  </si>
-  <si>
-    <t>L_MODV2_SOIL_TKN_009</t>
-  </si>
-  <si>
-    <t>L_MODV2_SOIL_TKN_010</t>
-  </si>
-  <si>
-    <t>L_MODV2_SOIL_TKN_011</t>
-  </si>
-  <si>
-    <t>L_MODV2_SOIL_TKN_012</t>
-  </si>
-  <si>
-    <t>L_MODV2_SOIL_TKN_013</t>
-  </si>
-  <si>
-    <t>L_MODV2_SOIL_TKN_014</t>
   </si>
   <si>
     <t>S-TKN.19</t>
@@ -10224,7 +10219,7 @@
         <v>1107</v>
       </c>
       <c r="B570" t="s">
-        <v>1120</v>
+        <v>1744</v>
       </c>
     </row>
     <row r="571" spans="1:2" x14ac:dyDescent="0.25">
@@ -10232,7 +10227,7 @@
         <v>1109</v>
       </c>
       <c r="B571" t="s">
-        <v>1121</v>
+        <v>1745</v>
       </c>
     </row>
     <row r="572" spans="1:2" x14ac:dyDescent="0.25">
@@ -10240,7 +10235,7 @@
         <v>1111</v>
       </c>
       <c r="B572" t="s">
-        <v>1122</v>
+        <v>1746</v>
       </c>
     </row>
     <row r="573" spans="1:2" x14ac:dyDescent="0.25">
@@ -10248,7 +10243,7 @@
         <v>1113</v>
       </c>
       <c r="B573" t="s">
-        <v>1123</v>
+        <v>1747</v>
       </c>
     </row>
     <row r="574" spans="1:2" x14ac:dyDescent="0.25">
@@ -10256,7 +10251,7 @@
         <v>1115</v>
       </c>
       <c r="B574" t="s">
-        <v>1124</v>
+        <v>1745</v>
       </c>
     </row>
     <row r="575" spans="1:2" x14ac:dyDescent="0.25">
@@ -10264,7 +10259,7 @@
         <v>1117</v>
       </c>
       <c r="B575" t="s">
-        <v>1125</v>
+        <v>1746</v>
       </c>
     </row>
     <row r="576" spans="1:2" x14ac:dyDescent="0.25">
@@ -10272,303 +10267,303 @@
         <v>1119</v>
       </c>
       <c r="B576" t="s">
-        <v>1126</v>
+        <v>1744</v>
       </c>
     </row>
     <row r="577" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A577" t="s">
-        <v>1127</v>
+        <v>1120</v>
       </c>
       <c r="B577" t="s">
-        <v>1128</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="578" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A578" t="s">
-        <v>1129</v>
+        <v>1122</v>
       </c>
       <c r="B578" t="s">
-        <v>1130</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="579" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A579" t="s">
-        <v>1131</v>
+        <v>1124</v>
       </c>
       <c r="B579" t="s">
-        <v>1132</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="580" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A580" t="s">
-        <v>1133</v>
+        <v>1126</v>
       </c>
       <c r="B580" t="s">
-        <v>1134</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="581" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A581" s="7" t="s">
-        <v>1135</v>
+        <v>1128</v>
       </c>
       <c r="B581" t="s">
-        <v>1136</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="582" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A582" s="9" t="s">
-        <v>1137</v>
+        <v>1130</v>
       </c>
       <c r="B582" t="s">
-        <v>1138</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="583" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A583" s="4" t="s">
-        <v>1139</v>
+        <v>1132</v>
       </c>
       <c r="B583" t="s">
-        <v>1140</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="584" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A584" s="4" t="s">
-        <v>1141</v>
+        <v>1134</v>
       </c>
       <c r="B584" t="s">
-        <v>1142</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="585" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A585" s="7" t="s">
-        <v>1143</v>
+        <v>1136</v>
       </c>
       <c r="B585" t="s">
-        <v>1144</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="586" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A586" t="s">
-        <v>1145</v>
+        <v>1138</v>
       </c>
       <c r="B586" t="s">
-        <v>1146</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="587" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A587" s="9" t="s">
-        <v>1147</v>
+        <v>1140</v>
       </c>
       <c r="B587" t="s">
-        <v>1148</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="588" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A588" s="7" t="s">
-        <v>1149</v>
+        <v>1142</v>
       </c>
       <c r="B588" t="s">
-        <v>1150</v>
+        <v>1143</v>
       </c>
     </row>
     <row r="589" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A589" s="7" t="s">
-        <v>1151</v>
+        <v>1144</v>
       </c>
       <c r="B589" t="s">
-        <v>1152</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="590" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A590" s="9" t="s">
-        <v>1153</v>
+        <v>1146</v>
       </c>
       <c r="B590" t="s">
-        <v>1154</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="591" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A591" s="7" t="s">
-        <v>1155</v>
+        <v>1148</v>
       </c>
       <c r="B591" t="s">
-        <v>1156</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="592" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A592" s="7" t="s">
-        <v>1157</v>
+        <v>1150</v>
       </c>
       <c r="B592" t="s">
-        <v>1158</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="593" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A593" s="7" t="s">
-        <v>1159</v>
+        <v>1152</v>
       </c>
       <c r="B593" t="s">
-        <v>1160</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="594" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A594" s="7" t="s">
-        <v>1161</v>
+        <v>1154</v>
       </c>
       <c r="B594" t="s">
-        <v>1162</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="595" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A595" s="7" t="s">
-        <v>1163</v>
+        <v>1156</v>
       </c>
       <c r="B595" t="s">
-        <v>1164</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="596" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A596" s="6" t="s">
-        <v>1165</v>
+        <v>1158</v>
       </c>
       <c r="B596" t="s">
-        <v>1166</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="597" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A597" s="6" t="s">
-        <v>1167</v>
+        <v>1160</v>
       </c>
       <c r="B597" t="s">
-        <v>1168</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="598" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A598" t="s">
-        <v>1169</v>
+        <v>1162</v>
       </c>
       <c r="B598" t="s">
-        <v>1170</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="599" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A599" s="6" t="s">
-        <v>1171</v>
+        <v>1164</v>
       </c>
       <c r="B599" t="s">
-        <v>1172</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="600" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A600" t="s">
-        <v>1173</v>
+        <v>1166</v>
       </c>
       <c r="B600" t="s">
-        <v>1174</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="601" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A601" s="6" t="s">
-        <v>1175</v>
+        <v>1168</v>
       </c>
       <c r="B601" t="s">
-        <v>1176</v>
+        <v>1169</v>
       </c>
     </row>
     <row r="602" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A602" t="s">
-        <v>1177</v>
+        <v>1170</v>
       </c>
       <c r="B602" t="s">
-        <v>1178</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="603" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A603" s="6" t="s">
-        <v>1179</v>
+        <v>1172</v>
       </c>
       <c r="B603" t="s">
-        <v>1180</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="604" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A604" s="6" t="s">
-        <v>1181</v>
+        <v>1174</v>
       </c>
       <c r="B604" t="s">
-        <v>1182</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="605" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A605" s="6" t="s">
-        <v>1183</v>
+        <v>1176</v>
       </c>
       <c r="B605" t="s">
-        <v>1184</v>
+        <v>1177</v>
       </c>
     </row>
     <row r="606" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A606" t="s">
-        <v>1185</v>
+        <v>1178</v>
       </c>
       <c r="B606" t="s">
-        <v>1186</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="607" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A607" s="6" t="s">
-        <v>1187</v>
+        <v>1180</v>
       </c>
       <c r="B607" t="s">
-        <v>1188</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="608" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A608" s="9" t="s">
-        <v>1189</v>
+        <v>1182</v>
       </c>
       <c r="B608" t="s">
-        <v>1190</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="609" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A609" t="s">
-        <v>1191</v>
+        <v>1184</v>
       </c>
       <c r="B609" t="s">
-        <v>1192</v>
+        <v>1185</v>
       </c>
     </row>
     <row r="610" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A610" s="4" t="s">
-        <v>1193</v>
+        <v>1186</v>
       </c>
       <c r="B610" t="s">
-        <v>1194</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="611" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A611" s="9" t="s">
-        <v>1195</v>
+        <v>1188</v>
       </c>
       <c r="B611" t="s">
-        <v>1196</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="612" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A612" s="9" t="s">
-        <v>1197</v>
+        <v>1190</v>
       </c>
       <c r="B612" t="s">
-        <v>1198</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="613" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A613" t="s">
-        <v>1199</v>
+        <v>1192</v>
       </c>
       <c r="B613" t="s">
-        <v>1200</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="614" spans="1:2" x14ac:dyDescent="0.25">
@@ -10576,7 +10571,7 @@
         <v>534</v>
       </c>
       <c r="B614" t="s">
-        <v>1201</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="615" spans="1:2" x14ac:dyDescent="0.25">
@@ -10584,15 +10579,15 @@
         <v>955</v>
       </c>
       <c r="B615" t="s">
-        <v>1202</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="616" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A616" t="s">
-        <v>1203</v>
+        <v>1196</v>
       </c>
       <c r="B616" t="s">
-        <v>1204</v>
+        <v>1197</v>
       </c>
     </row>
     <row r="617" spans="1:2" x14ac:dyDescent="0.25">
@@ -10600,7 +10595,7 @@
         <v>9</v>
       </c>
       <c r="B617" t="s">
-        <v>1205</v>
+        <v>1198</v>
       </c>
     </row>
     <row r="618" spans="1:2" x14ac:dyDescent="0.25">
@@ -10608,7 +10603,7 @@
         <v>13</v>
       </c>
       <c r="B618" t="s">
-        <v>1206</v>
+        <v>1199</v>
       </c>
     </row>
     <row r="619" spans="1:2" x14ac:dyDescent="0.25">
@@ -10616,31 +10611,31 @@
         <v>17</v>
       </c>
       <c r="B619" t="s">
-        <v>1207</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="620" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A620" t="s">
-        <v>1208</v>
+        <v>1201</v>
       </c>
       <c r="B620" t="s">
-        <v>1209</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="621" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A621" t="s">
-        <v>1210</v>
+        <v>1203</v>
       </c>
       <c r="B621" t="s">
-        <v>1211</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="622" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A622" t="s">
-        <v>1212</v>
+        <v>1205</v>
       </c>
       <c r="B622" t="s">
-        <v>1213</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="623" spans="1:2" x14ac:dyDescent="0.25">
@@ -10648,7 +10643,7 @@
         <v>19</v>
       </c>
       <c r="B623" t="s">
-        <v>1214</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="624" spans="1:2" x14ac:dyDescent="0.25">
@@ -10656,7 +10651,7 @@
         <v>21</v>
       </c>
       <c r="B624" t="s">
-        <v>1215</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="625" spans="1:2" x14ac:dyDescent="0.25">
@@ -10664,7 +10659,7 @@
         <v>23</v>
       </c>
       <c r="B625" t="s">
-        <v>1216</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="626" spans="1:2" x14ac:dyDescent="0.25">
@@ -10672,15 +10667,15 @@
         <v>27</v>
       </c>
       <c r="B626" t="s">
-        <v>1217</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="627" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A627" t="s">
-        <v>1218</v>
+        <v>1211</v>
       </c>
       <c r="B627" t="s">
-        <v>1219</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="628" spans="1:2" x14ac:dyDescent="0.25">
@@ -10688,39 +10683,39 @@
         <v>30</v>
       </c>
       <c r="B628" t="s">
-        <v>1220</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="629" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A629" t="s">
-        <v>1221</v>
+        <v>1214</v>
       </c>
       <c r="B629" t="s">
-        <v>1222</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="630" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A630" t="s">
-        <v>1223</v>
+        <v>1216</v>
       </c>
       <c r="B630" t="s">
-        <v>1224</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="631" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A631" t="s">
-        <v>1225</v>
+        <v>1218</v>
       </c>
       <c r="B631" t="s">
-        <v>1226</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="632" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A632" t="s">
-        <v>1227</v>
+        <v>1220</v>
       </c>
       <c r="B632" t="s">
-        <v>1228</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="633" spans="1:2" x14ac:dyDescent="0.25">
@@ -10728,15 +10723,15 @@
         <v>34</v>
       </c>
       <c r="B633" t="s">
-        <v>1229</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="634" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A634" t="s">
-        <v>1230</v>
+        <v>1223</v>
       </c>
       <c r="B634" t="s">
-        <v>1231</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="635" spans="1:2" x14ac:dyDescent="0.25">
@@ -10744,7 +10739,7 @@
         <v>722</v>
       </c>
       <c r="B635" t="s">
-        <v>1232</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="636" spans="1:2" x14ac:dyDescent="0.25">
@@ -10752,7 +10747,7 @@
         <v>724</v>
       </c>
       <c r="B636" t="s">
-        <v>1233</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="637" spans="1:2" x14ac:dyDescent="0.25">
@@ -10760,7 +10755,7 @@
         <v>726</v>
       </c>
       <c r="B637" t="s">
-        <v>1234</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="638" spans="1:2" x14ac:dyDescent="0.25">
@@ -10768,7 +10763,7 @@
         <v>728</v>
       </c>
       <c r="B638" t="s">
-        <v>1235</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="639" spans="1:2" x14ac:dyDescent="0.25">
@@ -10776,7 +10771,7 @@
         <v>731</v>
       </c>
       <c r="B639" t="s">
-        <v>1236</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="640" spans="1:2" x14ac:dyDescent="0.25">
@@ -10784,7 +10779,7 @@
         <v>733</v>
       </c>
       <c r="B640" t="s">
-        <v>1237</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="641" spans="1:2" x14ac:dyDescent="0.25">
@@ -10792,7 +10787,7 @@
         <v>735</v>
       </c>
       <c r="B641" t="s">
-        <v>1238</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="642" spans="1:2" x14ac:dyDescent="0.25">
@@ -10800,7 +10795,7 @@
         <v>1039</v>
       </c>
       <c r="B642" t="s">
-        <v>1239</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="643" spans="1:2" x14ac:dyDescent="0.25">
@@ -10808,7 +10803,7 @@
         <v>36</v>
       </c>
       <c r="B643" t="s">
-        <v>1240</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="644" spans="1:2" x14ac:dyDescent="0.25">
@@ -10816,7 +10811,7 @@
         <v>38</v>
       </c>
       <c r="B644" t="s">
-        <v>1241</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="645" spans="1:2" x14ac:dyDescent="0.25">
@@ -10824,31 +10819,31 @@
         <v>40</v>
       </c>
       <c r="B645" t="s">
-        <v>1242</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="646" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A646" t="s">
-        <v>1243</v>
+        <v>1236</v>
       </c>
       <c r="B646" t="s">
-        <v>1244</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="647" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A647" t="s">
-        <v>1245</v>
+        <v>1238</v>
       </c>
       <c r="B647" t="s">
-        <v>1246</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="648" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A648" t="s">
-        <v>1247</v>
+        <v>1240</v>
       </c>
       <c r="B648" t="s">
-        <v>1248</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="649" spans="1:2" x14ac:dyDescent="0.25">
@@ -10856,39 +10851,39 @@
         <v>74</v>
       </c>
       <c r="B649" t="s">
-        <v>1249</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="650" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A650" t="s">
-        <v>1250</v>
+        <v>1243</v>
       </c>
       <c r="B650" t="s">
-        <v>1251</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="651" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A651" t="s">
-        <v>1252</v>
+        <v>1245</v>
       </c>
       <c r="B651" t="s">
-        <v>1253</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="652" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A652" t="s">
-        <v>1254</v>
+        <v>1247</v>
       </c>
       <c r="B652" t="s">
-        <v>1255</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="653" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A653" t="s">
-        <v>1256</v>
+        <v>1249</v>
       </c>
       <c r="B653" t="s">
-        <v>1257</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="654" spans="1:2" x14ac:dyDescent="0.25">
@@ -10896,15 +10891,15 @@
         <v>44</v>
       </c>
       <c r="B654" t="s">
-        <v>1258</v>
+        <v>1251</v>
       </c>
     </row>
     <row r="655" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A655" t="s">
-        <v>1259</v>
+        <v>1252</v>
       </c>
       <c r="B655" t="s">
-        <v>1260</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="656" spans="1:2" x14ac:dyDescent="0.25">
@@ -10912,7 +10907,7 @@
         <v>46</v>
       </c>
       <c r="B656" t="s">
-        <v>1261</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="657" spans="1:2" x14ac:dyDescent="0.25">
@@ -10920,7 +10915,7 @@
         <v>48</v>
       </c>
       <c r="B657" t="s">
-        <v>1262</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="658" spans="1:2" x14ac:dyDescent="0.25">
@@ -10928,7 +10923,7 @@
         <v>50</v>
       </c>
       <c r="B658" t="s">
-        <v>1263</v>
+        <v>1256</v>
       </c>
     </row>
     <row r="659" spans="1:2" x14ac:dyDescent="0.25">
@@ -10936,7 +10931,7 @@
         <v>52</v>
       </c>
       <c r="B659" t="s">
-        <v>1264</v>
+        <v>1257</v>
       </c>
     </row>
     <row r="660" spans="1:2" x14ac:dyDescent="0.25">
@@ -10944,7 +10939,7 @@
         <v>54</v>
       </c>
       <c r="B660" t="s">
-        <v>1265</v>
+        <v>1258</v>
       </c>
     </row>
     <row r="661" spans="1:2" x14ac:dyDescent="0.25">
@@ -10952,7 +10947,7 @@
         <v>56</v>
       </c>
       <c r="B661" t="s">
-        <v>1266</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="662" spans="1:2" x14ac:dyDescent="0.25">
@@ -10960,7 +10955,7 @@
         <v>58</v>
       </c>
       <c r="B662" t="s">
-        <v>1267</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="663" spans="1:2" x14ac:dyDescent="0.25">
@@ -10968,7 +10963,7 @@
         <v>62</v>
       </c>
       <c r="B663" t="s">
-        <v>1268</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="664" spans="1:2" x14ac:dyDescent="0.25">
@@ -10976,23 +10971,23 @@
         <v>64</v>
       </c>
       <c r="B664" t="s">
-        <v>1269</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="665" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A665" t="s">
-        <v>1270</v>
+        <v>1263</v>
       </c>
       <c r="B665" t="s">
-        <v>1271</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="666" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A666" t="s">
-        <v>1272</v>
+        <v>1265</v>
       </c>
       <c r="B666" t="s">
-        <v>1273</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="667" spans="1:2" x14ac:dyDescent="0.25">
@@ -11000,7 +10995,7 @@
         <v>66</v>
       </c>
       <c r="B667" t="s">
-        <v>1274</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="668" spans="1:2" x14ac:dyDescent="0.25">
@@ -11008,7 +11003,7 @@
         <v>68</v>
       </c>
       <c r="B668" t="s">
-        <v>1275</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="669" spans="1:2" x14ac:dyDescent="0.25">
@@ -11016,23 +11011,23 @@
         <v>70</v>
       </c>
       <c r="B669" t="s">
-        <v>1276</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="670" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A670" t="s">
-        <v>1277</v>
+        <v>1270</v>
       </c>
       <c r="B670" t="s">
-        <v>1278</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="671" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A671" t="s">
-        <v>1279</v>
+        <v>1272</v>
       </c>
       <c r="B671" t="s">
-        <v>1280</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="672" spans="1:2" x14ac:dyDescent="0.25">
@@ -11040,7 +11035,7 @@
         <v>192</v>
       </c>
       <c r="B672" t="s">
-        <v>1281</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="673" spans="1:2" x14ac:dyDescent="0.25">
@@ -11048,39 +11043,39 @@
         <v>194</v>
       </c>
       <c r="B673" t="s">
-        <v>1282</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="674" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A674" t="s">
-        <v>1283</v>
+        <v>1276</v>
       </c>
       <c r="B674" t="s">
-        <v>1284</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="675" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A675" t="s">
-        <v>1285</v>
+        <v>1278</v>
       </c>
       <c r="B675" t="s">
-        <v>1286</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="676" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A676" t="s">
-        <v>1287</v>
+        <v>1280</v>
       </c>
       <c r="B676" t="s">
-        <v>1288</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="677" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A677" t="s">
-        <v>1289</v>
+        <v>1282</v>
       </c>
       <c r="B677" t="s">
-        <v>1290</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="678" spans="1:2" x14ac:dyDescent="0.25">
@@ -11088,7 +11083,7 @@
         <v>112</v>
       </c>
       <c r="B678" t="s">
-        <v>1291</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="679" spans="1:2" x14ac:dyDescent="0.25">
@@ -11096,15 +11091,15 @@
         <v>114</v>
       </c>
       <c r="B679" t="s">
-        <v>1292</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="680" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A680" t="s">
-        <v>1293</v>
+        <v>1286</v>
       </c>
       <c r="B680" t="s">
-        <v>1294</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="681" spans="1:2" x14ac:dyDescent="0.25">
@@ -11112,7 +11107,7 @@
         <v>124</v>
       </c>
       <c r="B681" t="s">
-        <v>1295</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="682" spans="1:2" x14ac:dyDescent="0.25">
@@ -11120,7 +11115,7 @@
         <v>128</v>
       </c>
       <c r="B682" t="s">
-        <v>1296</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="683" spans="1:2" x14ac:dyDescent="0.25">
@@ -11128,7 +11123,7 @@
         <v>130</v>
       </c>
       <c r="B683" t="s">
-        <v>1297</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="684" spans="1:2" x14ac:dyDescent="0.25">
@@ -11136,7 +11131,7 @@
         <v>132</v>
       </c>
       <c r="B684" t="s">
-        <v>1298</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="685" spans="1:2" x14ac:dyDescent="0.25">
@@ -11144,15 +11139,15 @@
         <v>134</v>
       </c>
       <c r="B685" t="s">
-        <v>1299</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="686" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A686" t="s">
-        <v>1300</v>
+        <v>1293</v>
       </c>
       <c r="B686" t="s">
-        <v>1301</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="687" spans="1:2" x14ac:dyDescent="0.25">
@@ -11160,7 +11155,7 @@
         <v>136</v>
       </c>
       <c r="B687" t="s">
-        <v>1302</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="688" spans="1:2" x14ac:dyDescent="0.25">
@@ -11168,7 +11163,7 @@
         <v>138</v>
       </c>
       <c r="B688" t="s">
-        <v>1303</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="689" spans="1:2" x14ac:dyDescent="0.25">
@@ -11176,7 +11171,7 @@
         <v>140</v>
       </c>
       <c r="B689" t="s">
-        <v>1304</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="690" spans="1:2" x14ac:dyDescent="0.25">
@@ -11184,7 +11179,7 @@
         <v>142</v>
       </c>
       <c r="B690" t="s">
-        <v>1305</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="691" spans="1:2" x14ac:dyDescent="0.25">
@@ -11192,7 +11187,7 @@
         <v>144</v>
       </c>
       <c r="B691" t="s">
-        <v>1306</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="692" spans="1:2" x14ac:dyDescent="0.25">
@@ -11200,7 +11195,7 @@
         <v>146</v>
       </c>
       <c r="B692" t="s">
-        <v>1307</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="693" spans="1:2" x14ac:dyDescent="0.25">
@@ -11208,7 +11203,7 @@
         <v>148</v>
       </c>
       <c r="B693" t="s">
-        <v>1308</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="694" spans="1:2" x14ac:dyDescent="0.25">
@@ -11216,15 +11211,15 @@
         <v>150</v>
       </c>
       <c r="B694" t="s">
-        <v>1309</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="695" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A695" t="s">
-        <v>1310</v>
+        <v>1303</v>
       </c>
       <c r="B695" t="s">
-        <v>1311</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="696" spans="1:2" x14ac:dyDescent="0.25">
@@ -11232,7 +11227,7 @@
         <v>156</v>
       </c>
       <c r="B696" t="s">
-        <v>1312</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="697" spans="1:2" x14ac:dyDescent="0.25">
@@ -11240,7 +11235,7 @@
         <v>160</v>
       </c>
       <c r="B697" t="s">
-        <v>1313</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="698" spans="1:2" x14ac:dyDescent="0.25">
@@ -11248,7 +11243,7 @@
         <v>108</v>
       </c>
       <c r="B698" t="s">
-        <v>1314</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="699" spans="1:2" x14ac:dyDescent="0.25">
@@ -11256,7 +11251,7 @@
         <v>262</v>
       </c>
       <c r="B699" t="s">
-        <v>1315</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="700" spans="1:2" x14ac:dyDescent="0.25">
@@ -11264,7 +11259,7 @@
         <v>264</v>
       </c>
       <c r="B700" t="s">
-        <v>1316</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="701" spans="1:2" x14ac:dyDescent="0.25">
@@ -11272,7 +11267,7 @@
         <v>266</v>
       </c>
       <c r="B701" t="s">
-        <v>1317</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="702" spans="1:2" x14ac:dyDescent="0.25">
@@ -11280,7 +11275,7 @@
         <v>268</v>
       </c>
       <c r="B702" t="s">
-        <v>1318</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="703" spans="1:2" x14ac:dyDescent="0.25">
@@ -11288,7 +11283,7 @@
         <v>270</v>
       </c>
       <c r="B703" t="s">
-        <v>1319</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="704" spans="1:2" x14ac:dyDescent="0.25">
@@ -11296,7 +11291,7 @@
         <v>272</v>
       </c>
       <c r="B704" t="s">
-        <v>1320</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="705" spans="1:2" x14ac:dyDescent="0.25">
@@ -11304,7 +11299,7 @@
         <v>274</v>
       </c>
       <c r="B705" t="s">
-        <v>1321</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="706" spans="1:2" x14ac:dyDescent="0.25">
@@ -11312,7 +11307,7 @@
         <v>276</v>
       </c>
       <c r="B706" t="s">
-        <v>1322</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="707" spans="1:2" x14ac:dyDescent="0.25">
@@ -11320,7 +11315,7 @@
         <v>278</v>
       </c>
       <c r="B707" t="s">
-        <v>1323</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="708" spans="1:2" x14ac:dyDescent="0.25">
@@ -11328,7 +11323,7 @@
         <v>280</v>
       </c>
       <c r="B708" t="s">
-        <v>1324</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="709" spans="1:2" x14ac:dyDescent="0.25">
@@ -11336,7 +11331,7 @@
         <v>282</v>
       </c>
       <c r="B709" t="s">
-        <v>1325</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="710" spans="1:2" x14ac:dyDescent="0.25">
@@ -11344,7 +11339,7 @@
         <v>284</v>
       </c>
       <c r="B710" t="s">
-        <v>1326</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="711" spans="1:2" x14ac:dyDescent="0.25">
@@ -11352,7 +11347,7 @@
         <v>286</v>
       </c>
       <c r="B711" t="s">
-        <v>1327</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="712" spans="1:2" x14ac:dyDescent="0.25">
@@ -11360,7 +11355,7 @@
         <v>288</v>
       </c>
       <c r="B712" t="s">
-        <v>1328</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="713" spans="1:2" x14ac:dyDescent="0.25">
@@ -11368,7 +11363,7 @@
         <v>291</v>
       </c>
       <c r="B713" t="s">
-        <v>1329</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="714" spans="1:2" x14ac:dyDescent="0.25">
@@ -11376,15 +11371,15 @@
         <v>293</v>
       </c>
       <c r="B714" t="s">
-        <v>1330</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="715" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A715" t="s">
-        <v>1331</v>
+        <v>1324</v>
       </c>
       <c r="B715" t="s">
-        <v>1332</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="716" spans="1:2" x14ac:dyDescent="0.25">
@@ -11392,7 +11387,7 @@
         <v>198</v>
       </c>
       <c r="B716" t="s">
-        <v>1333</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="717" spans="1:2" x14ac:dyDescent="0.25">
@@ -11400,7 +11395,7 @@
         <v>200</v>
       </c>
       <c r="B717" t="s">
-        <v>1334</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="718" spans="1:2" x14ac:dyDescent="0.25">
@@ -11408,15 +11403,15 @@
         <v>202</v>
       </c>
       <c r="B718" t="s">
-        <v>1335</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="719" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A719" t="s">
-        <v>1336</v>
+        <v>1329</v>
       </c>
       <c r="B719" t="s">
-        <v>1337</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="720" spans="1:2" x14ac:dyDescent="0.25">
@@ -11424,7 +11419,7 @@
         <v>221</v>
       </c>
       <c r="B720" t="s">
-        <v>1338</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="721" spans="1:2" x14ac:dyDescent="0.25">
@@ -11432,7 +11427,7 @@
         <v>324</v>
       </c>
       <c r="B721" t="s">
-        <v>1339</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="722" spans="1:2" x14ac:dyDescent="0.25">
@@ -11440,31 +11435,31 @@
         <v>326</v>
       </c>
       <c r="B722" t="s">
-        <v>1340</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="723" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A723" t="s">
-        <v>1341</v>
+        <v>1334</v>
       </c>
       <c r="B723" t="s">
-        <v>1342</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="724" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A724" t="s">
-        <v>1343</v>
+        <v>1336</v>
       </c>
       <c r="B724" t="s">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="725" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A725" t="s">
-        <v>1345</v>
+        <v>1338</v>
       </c>
       <c r="B725" t="s">
-        <v>1346</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="726" spans="1:2" x14ac:dyDescent="0.25">
@@ -11472,15 +11467,15 @@
         <v>301</v>
       </c>
       <c r="B726" t="s">
-        <v>1347</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="727" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A727" t="s">
-        <v>1348</v>
+        <v>1341</v>
       </c>
       <c r="B727" t="s">
-        <v>1349</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="728" spans="1:2" x14ac:dyDescent="0.25">
@@ -11488,39 +11483,39 @@
         <v>307</v>
       </c>
       <c r="B728" t="s">
-        <v>1350</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="729" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A729" t="s">
-        <v>1351</v>
+        <v>1344</v>
       </c>
       <c r="B729" t="s">
-        <v>1352</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="730" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A730" t="s">
-        <v>1353</v>
+        <v>1346</v>
       </c>
       <c r="B730" t="s">
-        <v>1354</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="731" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A731" t="s">
-        <v>1355</v>
+        <v>1348</v>
       </c>
       <c r="B731" t="s">
-        <v>1356</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="732" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A732" t="s">
-        <v>1357</v>
+        <v>1350</v>
       </c>
       <c r="B732" t="s">
-        <v>1358</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="733" spans="1:2" x14ac:dyDescent="0.25">
@@ -11528,7 +11523,7 @@
         <v>332</v>
       </c>
       <c r="B733" t="s">
-        <v>1359</v>
+        <v>1352</v>
       </c>
     </row>
     <row r="734" spans="1:2" x14ac:dyDescent="0.25">
@@ -11536,7 +11531,7 @@
         <v>334</v>
       </c>
       <c r="B734" t="s">
-        <v>1360</v>
+        <v>1353</v>
       </c>
     </row>
     <row r="735" spans="1:2" x14ac:dyDescent="0.25">
@@ -11544,7 +11539,7 @@
         <v>336</v>
       </c>
       <c r="B735" t="s">
-        <v>1361</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="736" spans="1:2" x14ac:dyDescent="0.25">
@@ -11552,23 +11547,23 @@
         <v>338</v>
       </c>
       <c r="B736" t="s">
-        <v>1362</v>
+        <v>1355</v>
       </c>
     </row>
     <row r="737" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A737" t="s">
-        <v>1363</v>
+        <v>1356</v>
       </c>
       <c r="B737" t="s">
-        <v>1364</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="738" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A738" t="s">
-        <v>1365</v>
+        <v>1358</v>
       </c>
       <c r="B738" t="s">
-        <v>1366</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="739" spans="1:2" x14ac:dyDescent="0.25">
@@ -11576,7 +11571,7 @@
         <v>342</v>
       </c>
       <c r="B739" t="s">
-        <v>1367</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="740" spans="1:2" x14ac:dyDescent="0.25">
@@ -11584,7 +11579,7 @@
         <v>344</v>
       </c>
       <c r="B740" t="s">
-        <v>1368</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="741" spans="1:2" x14ac:dyDescent="0.25">
@@ -11592,7 +11587,7 @@
         <v>346</v>
       </c>
       <c r="B741" t="s">
-        <v>1369</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="742" spans="1:2" x14ac:dyDescent="0.25">
@@ -11600,7 +11595,7 @@
         <v>348</v>
       </c>
       <c r="B742" t="s">
-        <v>1370</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="743" spans="1:2" x14ac:dyDescent="0.25">
@@ -11608,7 +11603,7 @@
         <v>350</v>
       </c>
       <c r="B743" t="s">
-        <v>1371</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="744" spans="1:2" x14ac:dyDescent="0.25">
@@ -11616,23 +11611,23 @@
         <v>352</v>
       </c>
       <c r="B744" t="s">
-        <v>1372</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="745" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A745" t="s">
-        <v>1373</v>
+        <v>1366</v>
       </c>
       <c r="B745" t="s">
-        <v>1374</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="746" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A746" t="s">
-        <v>1375</v>
+        <v>1368</v>
       </c>
       <c r="B746" t="s">
-        <v>1376</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="747" spans="1:2" x14ac:dyDescent="0.25">
@@ -11640,23 +11635,23 @@
         <v>356</v>
       </c>
       <c r="B747" t="s">
-        <v>1377</v>
+        <v>1370</v>
       </c>
     </row>
     <row r="748" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A748" t="s">
-        <v>1378</v>
+        <v>1371</v>
       </c>
       <c r="B748" t="s">
-        <v>1379</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="749" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A749" t="s">
-        <v>1380</v>
+        <v>1373</v>
       </c>
       <c r="B749" t="s">
-        <v>1381</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="750" spans="1:2" x14ac:dyDescent="0.25">
@@ -11664,15 +11659,15 @@
         <v>382</v>
       </c>
       <c r="B750" t="s">
-        <v>1382</v>
+        <v>1375</v>
       </c>
     </row>
     <row r="751" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A751" t="s">
-        <v>1383</v>
+        <v>1376</v>
       </c>
       <c r="B751" t="s">
-        <v>1384</v>
+        <v>1377</v>
       </c>
     </row>
     <row r="752" spans="1:2" x14ac:dyDescent="0.25">
@@ -11680,7 +11675,7 @@
         <v>384</v>
       </c>
       <c r="B752" t="s">
-        <v>1385</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="753" spans="1:2" x14ac:dyDescent="0.25">
@@ -11688,7 +11683,7 @@
         <v>386</v>
       </c>
       <c r="B753" t="s">
-        <v>1386</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="754" spans="1:2" x14ac:dyDescent="0.25">
@@ -11696,7 +11691,7 @@
         <v>388</v>
       </c>
       <c r="B754" t="s">
-        <v>1387</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="755" spans="1:2" x14ac:dyDescent="0.25">
@@ -11704,23 +11699,23 @@
         <v>392</v>
       </c>
       <c r="B755" t="s">
-        <v>1388</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="756" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A756" t="s">
-        <v>1389</v>
+        <v>1382</v>
       </c>
       <c r="B756" t="s">
-        <v>1390</v>
+        <v>1383</v>
       </c>
     </row>
     <row r="757" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A757" t="s">
-        <v>1391</v>
+        <v>1384</v>
       </c>
       <c r="B757" t="s">
-        <v>1392</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="758" spans="1:2" x14ac:dyDescent="0.25">
@@ -11728,7 +11723,7 @@
         <v>394</v>
       </c>
       <c r="B758" t="s">
-        <v>1393</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="759" spans="1:2" x14ac:dyDescent="0.25">
@@ -11736,7 +11731,7 @@
         <v>396</v>
       </c>
       <c r="B759" t="s">
-        <v>1394</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="760" spans="1:2" x14ac:dyDescent="0.25">
@@ -11744,7 +11739,7 @@
         <v>398</v>
       </c>
       <c r="B760" t="s">
-        <v>1395</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="761" spans="1:2" x14ac:dyDescent="0.25">
@@ -11752,7 +11747,7 @@
         <v>400</v>
       </c>
       <c r="B761" t="s">
-        <v>1396</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="762" spans="1:2" x14ac:dyDescent="0.25">
@@ -11760,7 +11755,7 @@
         <v>402</v>
       </c>
       <c r="B762" t="s">
-        <v>1397</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="763" spans="1:2" x14ac:dyDescent="0.25">
@@ -11768,15 +11763,15 @@
         <v>404</v>
       </c>
       <c r="B763" t="s">
-        <v>1398</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="764" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A764" t="s">
-        <v>1399</v>
+        <v>1392</v>
       </c>
       <c r="B764" t="s">
-        <v>1400</v>
+        <v>1393</v>
       </c>
     </row>
     <row r="765" spans="1:2" x14ac:dyDescent="0.25">
@@ -11784,7 +11779,7 @@
         <v>885</v>
       </c>
       <c r="B765" t="s">
-        <v>1401</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="766" spans="1:2" x14ac:dyDescent="0.25">
@@ -11792,7 +11787,7 @@
         <v>887</v>
       </c>
       <c r="B766" t="s">
-        <v>1402</v>
+        <v>1395</v>
       </c>
     </row>
     <row r="767" spans="1:2" x14ac:dyDescent="0.25">
@@ -11800,31 +11795,31 @@
         <v>889</v>
       </c>
       <c r="B767" t="s">
-        <v>1403</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="768" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A768" t="s">
-        <v>1404</v>
+        <v>1397</v>
       </c>
       <c r="B768" t="s">
-        <v>1405</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="769" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A769" t="s">
-        <v>1406</v>
+        <v>1399</v>
       </c>
       <c r="B769" t="s">
-        <v>1407</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="770" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A770" t="s">
-        <v>1408</v>
+        <v>1401</v>
       </c>
       <c r="B770" t="s">
-        <v>1409</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="771" spans="1:2" x14ac:dyDescent="0.25">
@@ -11832,7 +11827,7 @@
         <v>538</v>
       </c>
       <c r="B771" t="s">
-        <v>1410</v>
+        <v>1403</v>
       </c>
     </row>
     <row r="772" spans="1:2" x14ac:dyDescent="0.25">
@@ -11840,15 +11835,15 @@
         <v>562</v>
       </c>
       <c r="B772" t="s">
-        <v>1411</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="773" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A773" t="s">
-        <v>1412</v>
+        <v>1405</v>
       </c>
       <c r="B773" t="s">
-        <v>1413</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="774" spans="1:2" x14ac:dyDescent="0.25">
@@ -11856,7 +11851,7 @@
         <v>571</v>
       </c>
       <c r="B774" t="s">
-        <v>1414</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="775" spans="1:2" x14ac:dyDescent="0.25">
@@ -11864,7 +11859,7 @@
         <v>575</v>
       </c>
       <c r="B775" t="s">
-        <v>1415</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="776" spans="1:2" x14ac:dyDescent="0.25">
@@ -11872,7 +11867,7 @@
         <v>577</v>
       </c>
       <c r="B776" t="s">
-        <v>1416</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="777" spans="1:2" x14ac:dyDescent="0.25">
@@ -11880,7 +11875,7 @@
         <v>579</v>
       </c>
       <c r="B777" t="s">
-        <v>1417</v>
+        <v>1410</v>
       </c>
     </row>
     <row r="778" spans="1:2" x14ac:dyDescent="0.25">
@@ -11888,23 +11883,23 @@
         <v>581</v>
       </c>
       <c r="B778" t="s">
-        <v>1418</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="779" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A779" t="s">
-        <v>1419</v>
+        <v>1412</v>
       </c>
       <c r="B779" t="s">
-        <v>1420</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="780" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A780" t="s">
-        <v>1421</v>
+        <v>1414</v>
       </c>
       <c r="B780" t="s">
-        <v>1422</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="781" spans="1:2" x14ac:dyDescent="0.25">
@@ -11912,15 +11907,15 @@
         <v>583</v>
       </c>
       <c r="B781" t="s">
-        <v>1423</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="782" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A782" t="s">
-        <v>1424</v>
+        <v>1417</v>
       </c>
       <c r="B782" t="s">
-        <v>1425</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="783" spans="1:2" x14ac:dyDescent="0.25">
@@ -11928,7 +11923,7 @@
         <v>585</v>
       </c>
       <c r="B783" t="s">
-        <v>1426</v>
+        <v>1419</v>
       </c>
     </row>
     <row r="784" spans="1:2" x14ac:dyDescent="0.25">
@@ -11936,7 +11931,7 @@
         <v>587</v>
       </c>
       <c r="B784" t="s">
-        <v>1427</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="785" spans="1:2" x14ac:dyDescent="0.25">
@@ -11944,7 +11939,7 @@
         <v>589</v>
       </c>
       <c r="B785" t="s">
-        <v>1428</v>
+        <v>1421</v>
       </c>
     </row>
     <row r="786" spans="1:2" x14ac:dyDescent="0.25">
@@ -11952,7 +11947,7 @@
         <v>591</v>
       </c>
       <c r="B786" t="s">
-        <v>1429</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="787" spans="1:2" x14ac:dyDescent="0.25">
@@ -11960,7 +11955,7 @@
         <v>593</v>
       </c>
       <c r="B787" t="s">
-        <v>1430</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="788" spans="1:2" x14ac:dyDescent="0.25">
@@ -11968,7 +11963,7 @@
         <v>595</v>
       </c>
       <c r="B788" t="s">
-        <v>1431</v>
+        <v>1424</v>
       </c>
     </row>
     <row r="789" spans="1:2" x14ac:dyDescent="0.25">
@@ -11976,15 +11971,15 @@
         <v>597</v>
       </c>
       <c r="B789" t="s">
-        <v>1432</v>
+        <v>1425</v>
       </c>
     </row>
     <row r="790" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A790" t="s">
-        <v>1433</v>
+        <v>1426</v>
       </c>
       <c r="B790" t="s">
-        <v>1434</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="791" spans="1:2" x14ac:dyDescent="0.25">
@@ -11992,7 +11987,7 @@
         <v>603</v>
       </c>
       <c r="B791" t="s">
-        <v>1435</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="792" spans="1:2" x14ac:dyDescent="0.25">
@@ -12000,15 +11995,15 @@
         <v>607</v>
       </c>
       <c r="B792" t="s">
-        <v>1436</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="793" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A793" t="s">
-        <v>1437</v>
+        <v>1430</v>
       </c>
       <c r="B793" t="s">
-        <v>1438</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="794" spans="1:2" x14ac:dyDescent="0.25">
@@ -12016,7 +12011,7 @@
         <v>615</v>
       </c>
       <c r="B794" t="s">
-        <v>1439</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="795" spans="1:2" x14ac:dyDescent="0.25">
@@ -12024,7 +12019,7 @@
         <v>617</v>
       </c>
       <c r="B795" t="s">
-        <v>1440</v>
+        <v>1433</v>
       </c>
     </row>
     <row r="796" spans="1:2" x14ac:dyDescent="0.25">
@@ -12032,7 +12027,7 @@
         <v>619</v>
       </c>
       <c r="B796" t="s">
-        <v>1441</v>
+        <v>1434</v>
       </c>
     </row>
     <row r="797" spans="1:2" x14ac:dyDescent="0.25">
@@ -12040,31 +12035,31 @@
         <v>621</v>
       </c>
       <c r="B797" t="s">
-        <v>1442</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="798" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A798" t="s">
-        <v>1443</v>
+        <v>1436</v>
       </c>
       <c r="B798" t="s">
-        <v>1444</v>
+        <v>1437</v>
       </c>
     </row>
     <row r="799" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A799" t="s">
-        <v>1445</v>
+        <v>1438</v>
       </c>
       <c r="B799" t="s">
-        <v>1446</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="800" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A800" t="s">
-        <v>1447</v>
+        <v>1440</v>
       </c>
       <c r="B800" t="s">
-        <v>1448</v>
+        <v>1441</v>
       </c>
     </row>
     <row r="801" spans="1:2" x14ac:dyDescent="0.25">
@@ -12072,7 +12067,7 @@
         <v>623</v>
       </c>
       <c r="B801" t="s">
-        <v>1449</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="802" spans="1:2" x14ac:dyDescent="0.25">
@@ -12080,7 +12075,7 @@
         <v>625</v>
       </c>
       <c r="B802" t="s">
-        <v>1450</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="803" spans="1:2" x14ac:dyDescent="0.25">
@@ -12088,7 +12083,7 @@
         <v>627</v>
       </c>
       <c r="B803" t="s">
-        <v>1451</v>
+        <v>1444</v>
       </c>
     </row>
     <row r="804" spans="1:2" x14ac:dyDescent="0.25">
@@ -12096,7 +12091,7 @@
         <v>629</v>
       </c>
       <c r="B804" t="s">
-        <v>1452</v>
+        <v>1445</v>
       </c>
     </row>
     <row r="805" spans="1:2" x14ac:dyDescent="0.25">
@@ -12104,7 +12099,7 @@
         <v>631</v>
       </c>
       <c r="B805" t="s">
-        <v>1453</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="806" spans="1:2" x14ac:dyDescent="0.25">
@@ -12112,23 +12107,23 @@
         <v>633</v>
       </c>
       <c r="B806" t="s">
-        <v>1454</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="807" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A807" t="s">
-        <v>1455</v>
+        <v>1448</v>
       </c>
       <c r="B807" t="s">
-        <v>1456</v>
+        <v>1449</v>
       </c>
     </row>
     <row r="808" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A808" t="s">
-        <v>1457</v>
+        <v>1450</v>
       </c>
       <c r="B808" t="s">
-        <v>1458</v>
+        <v>1451</v>
       </c>
     </row>
     <row r="809" spans="1:2" x14ac:dyDescent="0.25">
@@ -12136,15 +12131,15 @@
         <v>637</v>
       </c>
       <c r="B809" t="s">
-        <v>1459</v>
+        <v>1452</v>
       </c>
     </row>
     <row r="810" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A810" t="s">
-        <v>1460</v>
+        <v>1453</v>
       </c>
       <c r="B810" t="s">
-        <v>1461</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="811" spans="1:2" x14ac:dyDescent="0.25">
@@ -12152,23 +12147,23 @@
         <v>445</v>
       </c>
       <c r="B811" t="s">
-        <v>1462</v>
+        <v>1455</v>
       </c>
     </row>
     <row r="812" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A812" t="s">
-        <v>1463</v>
+        <v>1456</v>
       </c>
       <c r="B812" t="s">
-        <v>1464</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="813" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A813" t="s">
-        <v>1465</v>
+        <v>1458</v>
       </c>
       <c r="B813" t="s">
-        <v>1466</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="814" spans="1:2" x14ac:dyDescent="0.25">
@@ -12176,15 +12171,15 @@
         <v>653</v>
       </c>
       <c r="B814" t="s">
-        <v>1467</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="815" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A815" t="s">
-        <v>1468</v>
+        <v>1461</v>
       </c>
       <c r="B815" t="s">
-        <v>1469</v>
+        <v>1462</v>
       </c>
     </row>
     <row r="816" spans="1:2" x14ac:dyDescent="0.25">
@@ -12192,15 +12187,15 @@
         <v>655</v>
       </c>
       <c r="B816" t="s">
-        <v>1470</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="817" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A817" t="s">
-        <v>1471</v>
+        <v>1464</v>
       </c>
       <c r="B817" t="s">
-        <v>1472</v>
+        <v>1465</v>
       </c>
     </row>
     <row r="818" spans="1:2" x14ac:dyDescent="0.25">
@@ -12208,7 +12203,7 @@
         <v>657</v>
       </c>
       <c r="B818" t="s">
-        <v>1473</v>
+        <v>1466</v>
       </c>
     </row>
     <row r="819" spans="1:2" x14ac:dyDescent="0.25">
@@ -12216,23 +12211,23 @@
         <v>659</v>
       </c>
       <c r="B819" t="s">
-        <v>1474</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="820" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A820" t="s">
-        <v>1475</v>
+        <v>1468</v>
       </c>
       <c r="B820" t="s">
-        <v>1476</v>
+        <v>1469</v>
       </c>
     </row>
     <row r="821" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A821" t="s">
-        <v>1477</v>
+        <v>1470</v>
       </c>
       <c r="B821" t="s">
-        <v>1478</v>
+        <v>1471</v>
       </c>
     </row>
     <row r="822" spans="1:2" x14ac:dyDescent="0.25">
@@ -12240,15 +12235,15 @@
         <v>661</v>
       </c>
       <c r="B822" t="s">
-        <v>1479</v>
+        <v>1472</v>
       </c>
     </row>
     <row r="823" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A823" t="s">
-        <v>1480</v>
+        <v>1473</v>
       </c>
       <c r="B823" t="s">
-        <v>1481</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="824" spans="1:2" x14ac:dyDescent="0.25">
@@ -12256,7 +12251,7 @@
         <v>663</v>
       </c>
       <c r="B824" t="s">
-        <v>1482</v>
+        <v>1475</v>
       </c>
     </row>
     <row r="825" spans="1:2" x14ac:dyDescent="0.25">
@@ -12264,7 +12259,7 @@
         <v>665</v>
       </c>
       <c r="B825" t="s">
-        <v>1483</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="826" spans="1:2" x14ac:dyDescent="0.25">
@@ -12272,15 +12267,15 @@
         <v>667</v>
       </c>
       <c r="B826" t="s">
-        <v>1484</v>
+        <v>1477</v>
       </c>
     </row>
     <row r="827" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A827" t="s">
-        <v>1485</v>
+        <v>1478</v>
       </c>
       <c r="B827" t="s">
-        <v>1486</v>
+        <v>1479</v>
       </c>
     </row>
     <row r="828" spans="1:2" x14ac:dyDescent="0.25">
@@ -12288,31 +12283,31 @@
         <v>741</v>
       </c>
       <c r="B828" t="s">
-        <v>1487</v>
+        <v>1480</v>
       </c>
     </row>
     <row r="829" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A829" t="s">
-        <v>1488</v>
+        <v>1481</v>
       </c>
       <c r="B829" t="s">
-        <v>1489</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="830" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A830" t="s">
-        <v>1490</v>
+        <v>1483</v>
       </c>
       <c r="B830" t="s">
-        <v>1491</v>
+        <v>1484</v>
       </c>
     </row>
     <row r="831" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A831" t="s">
-        <v>1492</v>
+        <v>1485</v>
       </c>
       <c r="B831" t="s">
-        <v>1493</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="832" spans="1:2" x14ac:dyDescent="0.25">
@@ -12320,23 +12315,23 @@
         <v>745</v>
       </c>
       <c r="B832" t="s">
-        <v>1494</v>
+        <v>1487</v>
       </c>
     </row>
     <row r="833" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A833" t="s">
-        <v>1495</v>
+        <v>1488</v>
       </c>
       <c r="B833" t="s">
-        <v>1496</v>
+        <v>1489</v>
       </c>
     </row>
     <row r="834" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A834" t="s">
-        <v>1497</v>
+        <v>1490</v>
       </c>
       <c r="B834" t="s">
-        <v>1498</v>
+        <v>1491</v>
       </c>
     </row>
     <row r="835" spans="1:2" x14ac:dyDescent="0.25">
@@ -12344,7 +12339,7 @@
         <v>747</v>
       </c>
       <c r="B835" t="s">
-        <v>1499</v>
+        <v>1492</v>
       </c>
     </row>
     <row r="836" spans="1:2" x14ac:dyDescent="0.25">
@@ -12352,7 +12347,7 @@
         <v>755</v>
       </c>
       <c r="B836" t="s">
-        <v>1500</v>
+        <v>1493</v>
       </c>
     </row>
     <row r="837" spans="1:2" x14ac:dyDescent="0.25">
@@ -12360,7 +12355,7 @@
         <v>757</v>
       </c>
       <c r="B837" t="s">
-        <v>1501</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="838" spans="1:2" x14ac:dyDescent="0.25">
@@ -12368,7 +12363,7 @@
         <v>759</v>
       </c>
       <c r="B838" t="s">
-        <v>1502</v>
+        <v>1495</v>
       </c>
     </row>
     <row r="839" spans="1:2" x14ac:dyDescent="0.25">
@@ -12376,7 +12371,7 @@
         <v>761</v>
       </c>
       <c r="B839" t="s">
-        <v>1503</v>
+        <v>1496</v>
       </c>
     </row>
     <row r="840" spans="1:2" x14ac:dyDescent="0.25">
@@ -12384,7 +12379,7 @@
         <v>763</v>
       </c>
       <c r="B840" t="s">
-        <v>1504</v>
+        <v>1497</v>
       </c>
     </row>
     <row r="841" spans="1:2" x14ac:dyDescent="0.25">
@@ -12392,7 +12387,7 @@
         <v>765</v>
       </c>
       <c r="B841" t="s">
-        <v>1505</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="842" spans="1:2" x14ac:dyDescent="0.25">
@@ -12400,7 +12395,7 @@
         <v>767</v>
       </c>
       <c r="B842" t="s">
-        <v>1506</v>
+        <v>1499</v>
       </c>
     </row>
     <row r="843" spans="1:2" x14ac:dyDescent="0.25">
@@ -12408,7 +12403,7 @@
         <v>769</v>
       </c>
       <c r="B843" t="s">
-        <v>1507</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="844" spans="1:2" x14ac:dyDescent="0.25">
@@ -12416,7 +12411,7 @@
         <v>771</v>
       </c>
       <c r="B844" t="s">
-        <v>1508</v>
+        <v>1501</v>
       </c>
     </row>
     <row r="845" spans="1:2" x14ac:dyDescent="0.25">
@@ -12424,7 +12419,7 @@
         <v>773</v>
       </c>
       <c r="B845" t="s">
-        <v>1509</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="846" spans="1:2" x14ac:dyDescent="0.25">
@@ -12432,7 +12427,7 @@
         <v>781</v>
       </c>
       <c r="B846" t="s">
-        <v>1510</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="847" spans="1:2" x14ac:dyDescent="0.25">
@@ -12440,31 +12435,31 @@
         <v>743</v>
       </c>
       <c r="B847" t="s">
-        <v>1511</v>
+        <v>1504</v>
       </c>
     </row>
     <row r="848" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A848" t="s">
-        <v>1512</v>
+        <v>1505</v>
       </c>
       <c r="B848" t="s">
-        <v>1513</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="849" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A849" t="s">
-        <v>1134</v>
+        <v>1127</v>
       </c>
       <c r="B849" t="s">
-        <v>1514</v>
+        <v>1507</v>
       </c>
     </row>
     <row r="850" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A850" t="s">
-        <v>1515</v>
+        <v>1508</v>
       </c>
       <c r="B850" t="s">
-        <v>1516</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="851" spans="1:2" x14ac:dyDescent="0.25">
@@ -12472,47 +12467,47 @@
         <v>647</v>
       </c>
       <c r="B851" t="s">
-        <v>1517</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="852" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A852" t="s">
-        <v>1518</v>
+        <v>1511</v>
       </c>
       <c r="B852" t="s">
-        <v>1519</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="853" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A853" t="s">
-        <v>1520</v>
+        <v>1513</v>
       </c>
       <c r="B853" t="s">
-        <v>1521</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="854" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A854" t="s">
-        <v>1522</v>
+        <v>1515</v>
       </c>
       <c r="B854" t="s">
-        <v>1523</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="855" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A855" t="s">
-        <v>1524</v>
+        <v>1517</v>
       </c>
       <c r="B855" t="s">
-        <v>1525</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="856" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A856" t="s">
-        <v>1526</v>
+        <v>1519</v>
       </c>
       <c r="B856" t="s">
-        <v>1527</v>
+        <v>1520</v>
       </c>
     </row>
     <row r="857" spans="1:2" x14ac:dyDescent="0.25">
@@ -12520,15 +12515,15 @@
         <v>812</v>
       </c>
       <c r="B857" t="s">
-        <v>1528</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="858" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A858" t="s">
-        <v>1529</v>
+        <v>1522</v>
       </c>
       <c r="B858" t="s">
-        <v>1530</v>
+        <v>1523</v>
       </c>
     </row>
     <row r="859" spans="1:2" x14ac:dyDescent="0.25">
@@ -12536,7 +12531,7 @@
         <v>814</v>
       </c>
       <c r="B859" t="s">
-        <v>1531</v>
+        <v>1524</v>
       </c>
     </row>
     <row r="860" spans="1:2" x14ac:dyDescent="0.25">
@@ -12544,7 +12539,7 @@
         <v>816</v>
       </c>
       <c r="B860" t="s">
-        <v>1532</v>
+        <v>1525</v>
       </c>
     </row>
     <row r="861" spans="1:2" x14ac:dyDescent="0.25">
@@ -12552,7 +12547,7 @@
         <v>818</v>
       </c>
       <c r="B861" t="s">
-        <v>1533</v>
+        <v>1526</v>
       </c>
     </row>
     <row r="862" spans="1:2" x14ac:dyDescent="0.25">
@@ -12560,7 +12555,7 @@
         <v>820</v>
       </c>
       <c r="B862" t="s">
-        <v>1534</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="863" spans="1:2" x14ac:dyDescent="0.25">
@@ -12568,7 +12563,7 @@
         <v>826</v>
       </c>
       <c r="B863" t="s">
-        <v>1535</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="864" spans="1:2" x14ac:dyDescent="0.25">
@@ -12576,7 +12571,7 @@
         <v>828</v>
       </c>
       <c r="B864" t="s">
-        <v>1536</v>
+        <v>1529</v>
       </c>
     </row>
     <row r="865" spans="1:2" x14ac:dyDescent="0.25">
@@ -12584,15 +12579,15 @@
         <v>830</v>
       </c>
       <c r="B865" t="s">
-        <v>1537</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="866" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A866" t="s">
-        <v>1538</v>
+        <v>1531</v>
       </c>
       <c r="B866" t="s">
-        <v>1539</v>
+        <v>1532</v>
       </c>
     </row>
     <row r="867" spans="1:2" x14ac:dyDescent="0.25">
@@ -12600,7 +12595,7 @@
         <v>832</v>
       </c>
       <c r="B867" t="s">
-        <v>1540</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="868" spans="1:2" x14ac:dyDescent="0.25">
@@ -12608,7 +12603,7 @@
         <v>835</v>
       </c>
       <c r="B868" t="s">
-        <v>1541</v>
+        <v>1534</v>
       </c>
     </row>
     <row r="869" spans="1:2" x14ac:dyDescent="0.25">
@@ -12616,7 +12611,7 @@
         <v>838</v>
       </c>
       <c r="B869" t="s">
-        <v>1542</v>
+        <v>1535</v>
       </c>
     </row>
     <row r="870" spans="1:2" x14ac:dyDescent="0.25">
@@ -12624,7 +12619,7 @@
         <v>840</v>
       </c>
       <c r="B870" t="s">
-        <v>1543</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="871" spans="1:2" x14ac:dyDescent="0.25">
@@ -12632,7 +12627,7 @@
         <v>842</v>
       </c>
       <c r="B871" t="s">
-        <v>1544</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="872" spans="1:2" x14ac:dyDescent="0.25">
@@ -12640,7 +12635,7 @@
         <v>844</v>
       </c>
       <c r="B872" t="s">
-        <v>1545</v>
+        <v>1538</v>
       </c>
     </row>
     <row r="873" spans="1:2" x14ac:dyDescent="0.25">
@@ -12648,7 +12643,7 @@
         <v>846</v>
       </c>
       <c r="B873" t="s">
-        <v>1546</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="874" spans="1:2" x14ac:dyDescent="0.25">
@@ -12656,7 +12651,7 @@
         <v>848</v>
       </c>
       <c r="B874" t="s">
-        <v>1547</v>
+        <v>1540</v>
       </c>
     </row>
     <row r="875" spans="1:2" x14ac:dyDescent="0.25">
@@ -12664,7 +12659,7 @@
         <v>850</v>
       </c>
       <c r="B875" t="s">
-        <v>1548</v>
+        <v>1541</v>
       </c>
     </row>
     <row r="876" spans="1:2" x14ac:dyDescent="0.25">
@@ -12672,7 +12667,7 @@
         <v>852</v>
       </c>
       <c r="B876" t="s">
-        <v>1549</v>
+        <v>1542</v>
       </c>
     </row>
     <row r="877" spans="1:2" x14ac:dyDescent="0.25">
@@ -12680,7 +12675,7 @@
         <v>854</v>
       </c>
       <c r="B877" t="s">
-        <v>1550</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="878" spans="1:2" x14ac:dyDescent="0.25">
@@ -12688,7 +12683,7 @@
         <v>856</v>
       </c>
       <c r="B878" t="s">
-        <v>1551</v>
+        <v>1544</v>
       </c>
     </row>
     <row r="879" spans="1:2" x14ac:dyDescent="0.25">
@@ -12696,7 +12691,7 @@
         <v>858</v>
       </c>
       <c r="B879" t="s">
-        <v>1552</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="880" spans="1:2" x14ac:dyDescent="0.25">
@@ -12704,23 +12699,23 @@
         <v>860</v>
       </c>
       <c r="B880" t="s">
-        <v>1553</v>
+        <v>1546</v>
       </c>
     </row>
     <row r="881" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A881" t="s">
-        <v>1554</v>
+        <v>1547</v>
       </c>
       <c r="B881" t="s">
-        <v>1555</v>
+        <v>1548</v>
       </c>
     </row>
     <row r="882" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A882" t="s">
-        <v>1556</v>
+        <v>1549</v>
       </c>
       <c r="B882" t="s">
-        <v>1557</v>
+        <v>1550</v>
       </c>
     </row>
     <row r="883" spans="1:2" x14ac:dyDescent="0.25">
@@ -12728,7 +12723,7 @@
         <v>862</v>
       </c>
       <c r="B883" t="s">
-        <v>1558</v>
+        <v>1551</v>
       </c>
     </row>
     <row r="884" spans="1:2" x14ac:dyDescent="0.25">
@@ -12736,7 +12731,7 @@
         <v>864</v>
       </c>
       <c r="B884" t="s">
-        <v>1559</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="885" spans="1:2" x14ac:dyDescent="0.25">
@@ -12744,15 +12739,15 @@
         <v>866</v>
       </c>
       <c r="B885" t="s">
-        <v>1560</v>
+        <v>1553</v>
       </c>
     </row>
     <row r="886" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A886" t="s">
-        <v>1561</v>
+        <v>1554</v>
       </c>
       <c r="B886" t="s">
-        <v>1562</v>
+        <v>1555</v>
       </c>
     </row>
     <row r="887" spans="1:2" x14ac:dyDescent="0.25">
@@ -12760,7 +12755,7 @@
         <v>868</v>
       </c>
       <c r="B887" t="s">
-        <v>1563</v>
+        <v>1556</v>
       </c>
     </row>
     <row r="888" spans="1:2" x14ac:dyDescent="0.25">
@@ -12768,15 +12763,15 @@
         <v>870</v>
       </c>
       <c r="B888" t="s">
-        <v>1564</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="889" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A889" t="s">
-        <v>1565</v>
+        <v>1558</v>
       </c>
       <c r="B889" t="s">
-        <v>1566</v>
+        <v>1559</v>
       </c>
     </row>
     <row r="890" spans="1:2" x14ac:dyDescent="0.25">
@@ -12784,7 +12779,7 @@
         <v>874</v>
       </c>
       <c r="B890" t="s">
-        <v>1567</v>
+        <v>1560</v>
       </c>
     </row>
     <row r="891" spans="1:2" x14ac:dyDescent="0.25">
@@ -12792,7 +12787,7 @@
         <v>878</v>
       </c>
       <c r="B891" t="s">
-        <v>1568</v>
+        <v>1561</v>
       </c>
     </row>
     <row r="892" spans="1:2" x14ac:dyDescent="0.25">
@@ -12800,7 +12795,7 @@
         <v>881</v>
       </c>
       <c r="B892" t="s">
-        <v>1569</v>
+        <v>1562</v>
       </c>
     </row>
     <row r="893" spans="1:2" x14ac:dyDescent="0.25">
@@ -12808,15 +12803,15 @@
         <v>883</v>
       </c>
       <c r="B893" t="s">
-        <v>1570</v>
+        <v>1563</v>
       </c>
     </row>
     <row r="894" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A894" t="s">
-        <v>1571</v>
+        <v>1564</v>
       </c>
       <c r="B894" t="s">
-        <v>1572</v>
+        <v>1565</v>
       </c>
     </row>
     <row r="895" spans="1:2" x14ac:dyDescent="0.25">
@@ -12824,7 +12819,7 @@
         <v>891</v>
       </c>
       <c r="B895" t="s">
-        <v>1573</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="896" spans="1:2" x14ac:dyDescent="0.25">
@@ -12832,7 +12827,7 @@
         <v>893</v>
       </c>
       <c r="B896" t="s">
-        <v>1574</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="897" spans="1:2" x14ac:dyDescent="0.25">
@@ -12840,7 +12835,7 @@
         <v>895</v>
       </c>
       <c r="B897" t="s">
-        <v>1575</v>
+        <v>1568</v>
       </c>
     </row>
     <row r="898" spans="1:2" x14ac:dyDescent="0.25">
@@ -12848,7 +12843,7 @@
         <v>897</v>
       </c>
       <c r="B898" t="s">
-        <v>1576</v>
+        <v>1569</v>
       </c>
     </row>
     <row r="899" spans="1:2" x14ac:dyDescent="0.25">
@@ -12856,7 +12851,7 @@
         <v>903</v>
       </c>
       <c r="B899" t="s">
-        <v>1577</v>
+        <v>1570</v>
       </c>
     </row>
     <row r="900" spans="1:2" x14ac:dyDescent="0.25">
@@ -12864,7 +12859,7 @@
         <v>905</v>
       </c>
       <c r="B900" t="s">
-        <v>1578</v>
+        <v>1571</v>
       </c>
     </row>
     <row r="901" spans="1:2" x14ac:dyDescent="0.25">
@@ -12872,23 +12867,23 @@
         <v>933</v>
       </c>
       <c r="B901" t="s">
-        <v>1579</v>
+        <v>1572</v>
       </c>
     </row>
     <row r="902" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A902" t="s">
-        <v>1580</v>
+        <v>1573</v>
       </c>
       <c r="B902" t="s">
-        <v>1581</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="903" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A903" t="s">
-        <v>1582</v>
+        <v>1575</v>
       </c>
       <c r="B903" t="s">
-        <v>1583</v>
+        <v>1576</v>
       </c>
     </row>
     <row r="904" spans="1:2" x14ac:dyDescent="0.25">
@@ -12896,7 +12891,7 @@
         <v>945</v>
       </c>
       <c r="B904" t="s">
-        <v>1584</v>
+        <v>1577</v>
       </c>
     </row>
     <row r="905" spans="1:2" x14ac:dyDescent="0.25">
@@ -12904,7 +12899,7 @@
         <v>947</v>
       </c>
       <c r="B905" t="s">
-        <v>1585</v>
+        <v>1578</v>
       </c>
     </row>
     <row r="906" spans="1:2" x14ac:dyDescent="0.25">
@@ -12912,23 +12907,23 @@
         <v>949</v>
       </c>
       <c r="B906" t="s">
-        <v>1586</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="907" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A907" t="s">
-        <v>1140</v>
+        <v>1133</v>
       </c>
       <c r="B907" t="s">
-        <v>1587</v>
+        <v>1580</v>
       </c>
     </row>
     <row r="908" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A908" t="s">
-        <v>1142</v>
+        <v>1135</v>
       </c>
       <c r="B908" t="s">
-        <v>1588</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="909" spans="1:2" x14ac:dyDescent="0.25">
@@ -12936,15 +12931,15 @@
         <v>453</v>
       </c>
       <c r="B909" t="s">
-        <v>1589</v>
+        <v>1582</v>
       </c>
     </row>
     <row r="910" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A910" t="s">
-        <v>1590</v>
+        <v>1583</v>
       </c>
       <c r="B910" t="s">
-        <v>1591</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="911" spans="1:2" x14ac:dyDescent="0.25">
@@ -12952,55 +12947,55 @@
         <v>462</v>
       </c>
       <c r="B911" t="s">
-        <v>1592</v>
+        <v>1585</v>
       </c>
     </row>
     <row r="912" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A912" t="s">
-        <v>1593</v>
+        <v>1586</v>
       </c>
       <c r="B912" t="s">
-        <v>1594</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="913" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A913" t="s">
-        <v>1595</v>
+        <v>1588</v>
       </c>
       <c r="B913" t="s">
-        <v>1596</v>
+        <v>1589</v>
       </c>
     </row>
     <row r="914" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A914" t="s">
-        <v>1597</v>
+        <v>1590</v>
       </c>
       <c r="B914" t="s">
-        <v>1598</v>
+        <v>1591</v>
       </c>
     </row>
     <row r="915" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A915" t="s">
-        <v>1599</v>
+        <v>1592</v>
       </c>
       <c r="B915" t="s">
-        <v>1600</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="916" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A916" t="s">
-        <v>1601</v>
+        <v>1594</v>
       </c>
       <c r="B916" t="s">
-        <v>1602</v>
+        <v>1595</v>
       </c>
     </row>
     <row r="917" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A917" t="s">
-        <v>1603</v>
+        <v>1596</v>
       </c>
       <c r="B917" t="s">
-        <v>1604</v>
+        <v>1597</v>
       </c>
     </row>
     <row r="918" spans="1:2" x14ac:dyDescent="0.25">
@@ -13008,15 +13003,15 @@
         <v>464</v>
       </c>
       <c r="B918" t="s">
-        <v>1605</v>
+        <v>1598</v>
       </c>
     </row>
     <row r="919" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A919" t="s">
-        <v>1606</v>
+        <v>1599</v>
       </c>
       <c r="B919" t="s">
-        <v>1607</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="920" spans="1:2" x14ac:dyDescent="0.25">
@@ -13024,7 +13019,7 @@
         <v>466</v>
       </c>
       <c r="B920" t="s">
-        <v>1608</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="921" spans="1:2" x14ac:dyDescent="0.25">
@@ -13032,15 +13027,15 @@
         <v>468</v>
       </c>
       <c r="B921" t="s">
-        <v>1609</v>
+        <v>1602</v>
       </c>
     </row>
     <row r="922" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A922" t="s">
-        <v>1610</v>
+        <v>1603</v>
       </c>
       <c r="B922" t="s">
-        <v>1611</v>
+        <v>1604</v>
       </c>
     </row>
     <row r="923" spans="1:2" x14ac:dyDescent="0.25">
@@ -13048,15 +13043,15 @@
         <v>470</v>
       </c>
       <c r="B923" t="s">
-        <v>1612</v>
+        <v>1605</v>
       </c>
     </row>
     <row r="924" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A924" t="s">
-        <v>1613</v>
+        <v>1606</v>
       </c>
       <c r="B924" t="s">
-        <v>1614</v>
+        <v>1607</v>
       </c>
     </row>
     <row r="925" spans="1:2" x14ac:dyDescent="0.25">
@@ -13064,7 +13059,7 @@
         <v>476</v>
       </c>
       <c r="B925" t="s">
-        <v>1615</v>
+        <v>1608</v>
       </c>
     </row>
     <row r="926" spans="1:2" x14ac:dyDescent="0.25">
@@ -13072,15 +13067,15 @@
         <v>478</v>
       </c>
       <c r="B926" t="s">
-        <v>1616</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="927" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A927" t="s">
-        <v>1617</v>
+        <v>1610</v>
       </c>
       <c r="B927" t="s">
-        <v>1618</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="928" spans="1:2" x14ac:dyDescent="0.25">
@@ -13088,7 +13083,7 @@
         <v>480</v>
       </c>
       <c r="B928" t="s">
-        <v>1619</v>
+        <v>1612</v>
       </c>
     </row>
     <row r="929" spans="1:2" x14ac:dyDescent="0.25">
@@ -13096,7 +13091,7 @@
         <v>482</v>
       </c>
       <c r="B929" t="s">
-        <v>1620</v>
+        <v>1613</v>
       </c>
     </row>
     <row r="930" spans="1:2" x14ac:dyDescent="0.25">
@@ -13104,7 +13099,7 @@
         <v>487</v>
       </c>
       <c r="B930" t="s">
-        <v>1621</v>
+        <v>1614</v>
       </c>
     </row>
     <row r="931" spans="1:2" x14ac:dyDescent="0.25">
@@ -13112,7 +13107,7 @@
         <v>489</v>
       </c>
       <c r="B931" t="s">
-        <v>1622</v>
+        <v>1615</v>
       </c>
     </row>
     <row r="932" spans="1:2" x14ac:dyDescent="0.25">
@@ -13120,7 +13115,7 @@
         <v>491</v>
       </c>
       <c r="B932" t="s">
-        <v>1623</v>
+        <v>1616</v>
       </c>
     </row>
     <row r="933" spans="1:2" x14ac:dyDescent="0.25">
@@ -13128,7 +13123,7 @@
         <v>494</v>
       </c>
       <c r="B933" t="s">
-        <v>1624</v>
+        <v>1617</v>
       </c>
     </row>
     <row r="934" spans="1:2" x14ac:dyDescent="0.25">
@@ -13136,7 +13131,7 @@
         <v>496</v>
       </c>
       <c r="B934" t="s">
-        <v>1625</v>
+        <v>1618</v>
       </c>
     </row>
     <row r="935" spans="1:2" x14ac:dyDescent="0.25">
@@ -13144,7 +13139,7 @@
         <v>504</v>
       </c>
       <c r="B935" t="s">
-        <v>1626</v>
+        <v>1619</v>
       </c>
     </row>
     <row r="936" spans="1:2" x14ac:dyDescent="0.25">
@@ -13152,15 +13147,15 @@
         <v>508</v>
       </c>
       <c r="B936" t="s">
-        <v>1627</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="937" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A937" t="s">
-        <v>1628</v>
+        <v>1621</v>
       </c>
       <c r="B937" t="s">
-        <v>1629</v>
+        <v>1622</v>
       </c>
     </row>
     <row r="938" spans="1:2" x14ac:dyDescent="0.25">
@@ -13168,23 +13163,23 @@
         <v>510</v>
       </c>
       <c r="B938" t="s">
-        <v>1630</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="939" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A939" t="s">
-        <v>1631</v>
+        <v>1624</v>
       </c>
       <c r="B939" t="s">
-        <v>1632</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="940" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A940" t="s">
-        <v>1633</v>
+        <v>1626</v>
       </c>
       <c r="B940" t="s">
-        <v>1634</v>
+        <v>1627</v>
       </c>
     </row>
     <row r="941" spans="1:2" x14ac:dyDescent="0.25">
@@ -13192,15 +13187,15 @@
         <v>516</v>
       </c>
       <c r="B941" t="s">
-        <v>1635</v>
+        <v>1628</v>
       </c>
     </row>
     <row r="942" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A942" t="s">
-        <v>1636</v>
+        <v>1629</v>
       </c>
       <c r="B942" t="s">
-        <v>1637</v>
+        <v>1630</v>
       </c>
     </row>
     <row r="943" spans="1:2" x14ac:dyDescent="0.25">
@@ -13208,23 +13203,23 @@
         <v>1105</v>
       </c>
       <c r="B943" t="s">
-        <v>1638</v>
+        <v>1631</v>
       </c>
     </row>
     <row r="944" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A944" t="s">
-        <v>1639</v>
+        <v>1632</v>
       </c>
       <c r="B944" t="s">
-        <v>1640</v>
+        <v>1633</v>
       </c>
     </row>
     <row r="945" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A945" t="s">
-        <v>1641</v>
+        <v>1634</v>
       </c>
       <c r="B945" t="s">
-        <v>1642</v>
+        <v>1635</v>
       </c>
     </row>
     <row r="946" spans="1:2" x14ac:dyDescent="0.25">
@@ -13232,15 +13227,15 @@
         <v>1041</v>
       </c>
       <c r="B946" t="s">
-        <v>1643</v>
+        <v>1636</v>
       </c>
     </row>
     <row r="947" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A947" t="s">
-        <v>1644</v>
+        <v>1637</v>
       </c>
       <c r="B947" t="s">
-        <v>1645</v>
+        <v>1638</v>
       </c>
     </row>
     <row r="948" spans="1:2" x14ac:dyDescent="0.25">
@@ -13248,31 +13243,31 @@
         <v>1043</v>
       </c>
       <c r="B948" t="s">
-        <v>1646</v>
+        <v>1639</v>
       </c>
     </row>
     <row r="949" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A949" t="s">
-        <v>1647</v>
+        <v>1640</v>
       </c>
       <c r="B949" t="s">
-        <v>1648</v>
+        <v>1641</v>
       </c>
     </row>
     <row r="950" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A950" t="s">
-        <v>1649</v>
+        <v>1642</v>
       </c>
       <c r="B950" t="s">
-        <v>1650</v>
+        <v>1643</v>
       </c>
     </row>
     <row r="951" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A951" t="s">
-        <v>1651</v>
+        <v>1644</v>
       </c>
       <c r="B951" t="s">
-        <v>1652</v>
+        <v>1645</v>
       </c>
     </row>
     <row r="952" spans="1:2" x14ac:dyDescent="0.25">
@@ -13280,15 +13275,15 @@
         <v>1045</v>
       </c>
       <c r="B952" t="s">
-        <v>1653</v>
+        <v>1646</v>
       </c>
     </row>
     <row r="953" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A953" t="s">
-        <v>1654</v>
+        <v>1647</v>
       </c>
       <c r="B953" t="s">
-        <v>1655</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="954" spans="1:2" x14ac:dyDescent="0.25">
@@ -13296,7 +13291,7 @@
         <v>1047</v>
       </c>
       <c r="B954" t="s">
-        <v>1656</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="955" spans="1:2" x14ac:dyDescent="0.25">
@@ -13304,7 +13299,7 @@
         <v>1053</v>
       </c>
       <c r="B955" t="s">
-        <v>1657</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="956" spans="1:2" x14ac:dyDescent="0.25">
@@ -13312,7 +13307,7 @@
         <v>5</v>
       </c>
       <c r="B956" t="s">
-        <v>1658</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="957" spans="1:2" x14ac:dyDescent="0.25">
@@ -13320,15 +13315,15 @@
         <v>677</v>
       </c>
       <c r="B957" t="s">
-        <v>1659</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="958" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A958" t="s">
-        <v>1660</v>
+        <v>1653</v>
       </c>
       <c r="B958" t="s">
-        <v>1661</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="959" spans="1:2" x14ac:dyDescent="0.25">
@@ -13336,15 +13331,15 @@
         <v>686</v>
       </c>
       <c r="B959" t="s">
-        <v>1662</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="960" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A960" t="s">
-        <v>1663</v>
+        <v>1656</v>
       </c>
       <c r="B960" t="s">
-        <v>1664</v>
+        <v>1657</v>
       </c>
     </row>
     <row r="961" spans="1:2" x14ac:dyDescent="0.25">
@@ -13352,7 +13347,7 @@
         <v>688</v>
       </c>
       <c r="B961" t="s">
-        <v>1665</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="962" spans="1:2" x14ac:dyDescent="0.25">
@@ -13360,7 +13355,7 @@
         <v>690</v>
       </c>
       <c r="B962" t="s">
-        <v>1666</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="963" spans="1:2" x14ac:dyDescent="0.25">
@@ -13368,7 +13363,7 @@
         <v>694</v>
       </c>
       <c r="B963" t="s">
-        <v>1667</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="964" spans="1:2" x14ac:dyDescent="0.25">
@@ -13376,7 +13371,7 @@
         <v>696</v>
       </c>
       <c r="B964" t="s">
-        <v>1668</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="965" spans="1:2" x14ac:dyDescent="0.25">
@@ -13384,7 +13379,7 @@
         <v>698</v>
       </c>
       <c r="B965" t="s">
-        <v>1669</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="966" spans="1:2" x14ac:dyDescent="0.25">
@@ -13392,7 +13387,7 @@
         <v>702</v>
       </c>
       <c r="B966" t="s">
-        <v>1670</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="967" spans="1:2" x14ac:dyDescent="0.25">
@@ -13400,7 +13395,7 @@
         <v>706</v>
       </c>
       <c r="B967" t="s">
-        <v>1671</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="968" spans="1:2" x14ac:dyDescent="0.25">
@@ -13408,7 +13403,7 @@
         <v>1087</v>
       </c>
       <c r="B968" t="s">
-        <v>1672</v>
+        <v>1665</v>
       </c>
     </row>
     <row r="969" spans="1:2" x14ac:dyDescent="0.25">
@@ -13416,15 +13411,15 @@
         <v>1085</v>
       </c>
       <c r="B969" t="s">
-        <v>1673</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="970" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A970" t="s">
-        <v>1674</v>
+        <v>1667</v>
       </c>
       <c r="B970" t="s">
-        <v>1675</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="971" spans="1:2" x14ac:dyDescent="0.25">
@@ -13432,15 +13427,15 @@
         <v>1071</v>
       </c>
       <c r="B971" t="s">
-        <v>1676</v>
+        <v>1669</v>
       </c>
     </row>
     <row r="972" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A972" t="s">
-        <v>1677</v>
+        <v>1670</v>
       </c>
       <c r="B972" t="s">
-        <v>1678</v>
+        <v>1671</v>
       </c>
     </row>
     <row r="973" spans="1:2" x14ac:dyDescent="0.25">
@@ -13448,7 +13443,7 @@
         <v>1073</v>
       </c>
       <c r="B973" t="s">
-        <v>1679</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="974" spans="1:2" x14ac:dyDescent="0.25">
@@ -13456,7 +13451,7 @@
         <v>961</v>
       </c>
       <c r="B974" t="s">
-        <v>1680</v>
+        <v>1673</v>
       </c>
     </row>
     <row r="975" spans="1:2" x14ac:dyDescent="0.25">
@@ -13464,7 +13459,7 @@
         <v>963</v>
       </c>
       <c r="B975" t="s">
-        <v>1681</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="976" spans="1:2" x14ac:dyDescent="0.25">
@@ -13472,7 +13467,7 @@
         <v>965</v>
       </c>
       <c r="B976" t="s">
-        <v>1682</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="977" spans="1:2" x14ac:dyDescent="0.25">
@@ -13480,7 +13475,7 @@
         <v>967</v>
       </c>
       <c r="B977" t="s">
-        <v>1683</v>
+        <v>1676</v>
       </c>
     </row>
     <row r="978" spans="1:2" x14ac:dyDescent="0.25">
@@ -13488,15 +13483,15 @@
         <v>969</v>
       </c>
       <c r="B978" t="s">
-        <v>1684</v>
+        <v>1677</v>
       </c>
     </row>
     <row r="979" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A979" t="s">
-        <v>1685</v>
+        <v>1678</v>
       </c>
       <c r="B979" t="s">
-        <v>1686</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="980" spans="1:2" x14ac:dyDescent="0.25">
@@ -13504,15 +13499,15 @@
         <v>971</v>
       </c>
       <c r="B980" t="s">
-        <v>1687</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="981" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A981" t="s">
-        <v>1688</v>
+        <v>1681</v>
       </c>
       <c r="B981" t="s">
-        <v>1689</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="982" spans="1:2" x14ac:dyDescent="0.25">
@@ -13520,7 +13515,7 @@
         <v>975</v>
       </c>
       <c r="B982" t="s">
-        <v>1690</v>
+        <v>1683</v>
       </c>
     </row>
     <row r="983" spans="1:2" x14ac:dyDescent="0.25">
@@ -13528,7 +13523,7 @@
         <v>979</v>
       </c>
       <c r="B983" t="s">
-        <v>1691</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="984" spans="1:2" x14ac:dyDescent="0.25">
@@ -13536,15 +13531,15 @@
         <v>981</v>
       </c>
       <c r="B984" t="s">
-        <v>1692</v>
+        <v>1685</v>
       </c>
     </row>
     <row r="985" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A985" t="s">
-        <v>1693</v>
+        <v>1686</v>
       </c>
       <c r="B985" t="s">
-        <v>1694</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="986" spans="1:2" x14ac:dyDescent="0.25">
@@ -13552,7 +13547,7 @@
         <v>983</v>
       </c>
       <c r="B986" t="s">
-        <v>1695</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="987" spans="1:2" x14ac:dyDescent="0.25">
@@ -13560,7 +13555,7 @@
         <v>985</v>
       </c>
       <c r="B987" t="s">
-        <v>1696</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="988" spans="1:2" x14ac:dyDescent="0.25">
@@ -13568,31 +13563,31 @@
         <v>987</v>
       </c>
       <c r="B988" t="s">
-        <v>1697</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="989" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A989" t="s">
-        <v>1698</v>
+        <v>1691</v>
       </c>
       <c r="B989" t="s">
-        <v>1699</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="990" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A990" t="s">
-        <v>1700</v>
+        <v>1693</v>
       </c>
       <c r="B990" t="s">
-        <v>1701</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="991" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A991" t="s">
-        <v>1702</v>
+        <v>1695</v>
       </c>
       <c r="B991" t="s">
-        <v>1703</v>
+        <v>1696</v>
       </c>
     </row>
     <row r="992" spans="1:2" x14ac:dyDescent="0.25">
@@ -13600,15 +13595,15 @@
         <v>991</v>
       </c>
       <c r="B992" t="s">
-        <v>1704</v>
+        <v>1697</v>
       </c>
     </row>
     <row r="993" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A993" t="s">
-        <v>1705</v>
+        <v>1698</v>
       </c>
       <c r="B993" t="s">
-        <v>1706</v>
+        <v>1699</v>
       </c>
     </row>
     <row r="994" spans="1:2" x14ac:dyDescent="0.25">
@@ -13616,7 +13611,7 @@
         <v>993</v>
       </c>
       <c r="B994" t="s">
-        <v>1707</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="995" spans="1:2" x14ac:dyDescent="0.25">
@@ -13624,7 +13619,7 @@
         <v>997</v>
       </c>
       <c r="B995" t="s">
-        <v>1708</v>
+        <v>1701</v>
       </c>
     </row>
     <row r="996" spans="1:2" x14ac:dyDescent="0.25">
@@ -13632,15 +13627,15 @@
         <v>999</v>
       </c>
       <c r="B996" t="s">
-        <v>1709</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="997" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A997" t="s">
-        <v>1710</v>
+        <v>1703</v>
       </c>
       <c r="B997" t="s">
-        <v>1711</v>
+        <v>1704</v>
       </c>
     </row>
     <row r="998" spans="1:2" x14ac:dyDescent="0.25">
@@ -13648,7 +13643,7 @@
         <v>1007</v>
       </c>
       <c r="B998" t="s">
-        <v>1712</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="999" spans="1:2" x14ac:dyDescent="0.25">
@@ -13656,263 +13651,207 @@
         <v>1069</v>
       </c>
       <c r="B999" t="s">
-        <v>1713</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="1000" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1000" t="s">
-        <v>1714</v>
+        <v>1707</v>
       </c>
       <c r="B1000" t="s">
-        <v>1715</v>
+        <v>1708</v>
       </c>
     </row>
     <row r="1001" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1001" t="s">
-        <v>1716</v>
+        <v>1709</v>
       </c>
       <c r="B1001" t="s">
-        <v>1717</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="1002" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1002" t="s">
-        <v>1146</v>
+        <v>1139</v>
       </c>
       <c r="B1002" t="s">
-        <v>1718</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="1003" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1003" t="s">
-        <v>1719</v>
+        <v>1712</v>
       </c>
       <c r="B1003" t="s">
-        <v>1720</v>
+        <v>1713</v>
       </c>
     </row>
     <row r="1004" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1004" t="s">
-        <v>1721</v>
+        <v>1714</v>
       </c>
       <c r="B1004" t="s">
-        <v>1722</v>
+        <v>1715</v>
       </c>
     </row>
     <row r="1005" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1005" t="s">
-        <v>1723</v>
+        <v>1716</v>
       </c>
       <c r="B1005" t="s">
-        <v>1724</v>
+        <v>1717</v>
       </c>
     </row>
     <row r="1006" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1006" t="s">
-        <v>1725</v>
+        <v>1718</v>
       </c>
       <c r="B1006" t="s">
-        <v>1726</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="1007" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1007" t="s">
-        <v>1727</v>
+        <v>1720</v>
       </c>
       <c r="B1007" t="s">
-        <v>1728</v>
+        <v>1721</v>
       </c>
     </row>
     <row r="1008" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1008" t="s">
-        <v>1729</v>
+        <v>1722</v>
       </c>
       <c r="B1008" t="s">
-        <v>1730</v>
+        <v>1723</v>
       </c>
     </row>
     <row r="1009" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1009" t="s">
-        <v>1166</v>
+        <v>1159</v>
       </c>
       <c r="B1009" t="s">
-        <v>1731</v>
+        <v>1724</v>
       </c>
     </row>
     <row r="1010" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1010" t="s">
-        <v>1168</v>
+        <v>1161</v>
       </c>
       <c r="B1010" t="s">
-        <v>1732</v>
+        <v>1725</v>
       </c>
     </row>
     <row r="1011" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1011" t="s">
-        <v>1170</v>
+        <v>1163</v>
       </c>
       <c r="B1011" t="s">
-        <v>1733</v>
+        <v>1726</v>
       </c>
     </row>
     <row r="1012" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1012" t="s">
-        <v>1172</v>
+        <v>1165</v>
       </c>
       <c r="B1012" t="s">
-        <v>1734</v>
+        <v>1727</v>
       </c>
     </row>
     <row r="1013" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1013" t="s">
-        <v>1735</v>
+        <v>1728</v>
       </c>
       <c r="B1013" t="s">
-        <v>1736</v>
+        <v>1729</v>
       </c>
     </row>
     <row r="1014" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1014" t="s">
-        <v>1737</v>
+        <v>1730</v>
       </c>
       <c r="B1014" t="s">
-        <v>1738</v>
+        <v>1731</v>
       </c>
     </row>
     <row r="1015" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1015" t="s">
-        <v>1174</v>
+        <v>1167</v>
       </c>
       <c r="B1015" t="s">
-        <v>1739</v>
+        <v>1732</v>
       </c>
     </row>
     <row r="1016" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1016" t="s">
-        <v>1176</v>
+        <v>1169</v>
       </c>
       <c r="B1016" t="s">
-        <v>1740</v>
+        <v>1733</v>
       </c>
     </row>
     <row r="1017" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1017" t="s">
-        <v>1178</v>
+        <v>1171</v>
       </c>
       <c r="B1017" t="s">
-        <v>1741</v>
+        <v>1734</v>
       </c>
     </row>
     <row r="1018" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1018" t="s">
-        <v>1180</v>
+        <v>1173</v>
       </c>
       <c r="B1018" t="s">
-        <v>1742</v>
+        <v>1735</v>
       </c>
     </row>
     <row r="1019" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1019" t="s">
-        <v>1182</v>
+        <v>1175</v>
       </c>
       <c r="B1019" t="s">
-        <v>1743</v>
+        <v>1736</v>
       </c>
     </row>
     <row r="1020" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1020" t="s">
-        <v>1184</v>
+        <v>1177</v>
       </c>
       <c r="B1020" t="s">
-        <v>1744</v>
+        <v>1737</v>
       </c>
     </row>
     <row r="1021" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1021" t="s">
-        <v>1186</v>
+        <v>1179</v>
       </c>
       <c r="B1021" t="s">
-        <v>1745</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="1022" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1022" t="s">
-        <v>1188</v>
+        <v>1181</v>
       </c>
       <c r="B1022" t="s">
-        <v>1746</v>
+        <v>1739</v>
       </c>
     </row>
     <row r="1023" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1023" t="s">
-        <v>1747</v>
+        <v>1740</v>
       </c>
       <c r="B1023" t="s">
-        <v>1748</v>
+        <v>1741</v>
       </c>
     </row>
     <row r="1024" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1024" t="s">
-        <v>1749</v>
+        <v>1742</v>
       </c>
       <c r="B1024" t="s">
-        <v>1750</v>
-      </c>
-    </row>
-    <row r="1025" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1025" t="s">
-        <v>1120</v>
-      </c>
-      <c r="B1025" t="s">
-        <v>1751</v>
-      </c>
-    </row>
-    <row r="1026" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1026" t="s">
-        <v>1121</v>
-      </c>
-      <c r="B1026" t="s">
-        <v>1752</v>
-      </c>
-    </row>
-    <row r="1027" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1027" t="s">
-        <v>1122</v>
-      </c>
-      <c r="B1027" t="s">
-        <v>1753</v>
-      </c>
-    </row>
-    <row r="1028" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1028" t="s">
-        <v>1123</v>
-      </c>
-      <c r="B1028" t="s">
-        <v>1754</v>
-      </c>
-    </row>
-    <row r="1029" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1029" t="s">
-        <v>1124</v>
-      </c>
-      <c r="B1029" t="s">
-        <v>1752</v>
-      </c>
-    </row>
-    <row r="1030" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1030" t="s">
-        <v>1125</v>
-      </c>
-      <c r="B1030" t="s">
-        <v>1753</v>
-      </c>
-    </row>
-    <row r="1031" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1031" t="s">
-        <v>1126</v>
-      </c>
-      <c r="B1031" t="s">
-        <v>1751</v>
+        <v>1743</v>
       </c>
     </row>
     <row r="1032" spans="1:2" x14ac:dyDescent="0.25">
@@ -13920,10 +13859,11 @@
         <v>1101</v>
       </c>
       <c r="B1032" t="s">
-        <v>1755</v>
+        <v>1748</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B1032" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>